<commit_message>
corrección de la Z estandarización en regresion.
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Regre/DL_reg.xlsx
+++ b/modelado/modelos/resultados/Regre/DL_reg.xlsx
@@ -223,9 +223,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -251,9 +248,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -345,6 +339,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -370,6 +367,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1095,67 +1095,67 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0.577±0.009</t>
+          <t>0.574±0.008</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.762±0.006</t>
+          <t>0.759±0.005</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.846±0.036</t>
+          <t>0.842±0.013</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.552±0.008</t>
+          <t>0.548±0.007</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.693±0.018</t>
+          <t>1.700±0.015</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.170±0.002</t>
+          <t>0.171±0.002</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.120±0.032</t>
+          <t>1.121±0.023</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>-0.110±0.066</t>
+          <t>-0.095±0.054</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.714±0.059</t>
+          <t>0.710±0.030</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.721±0.005</t>
+          <t>0.719±0.004</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>56.722±1.020</t>
+          <t>57.093±1.156</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>55.567±0.949</t>
+          <t>55.722±0.782</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>38.554±1.004</t>
+          <t>38.983±0.803</t>
         </is>
       </c>
     </row>
@@ -1189,54 +1189,54 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vgo</t>
+          <t>mlotst</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.2586 ± 0.1685</t>
+          <t>0.0825 ± 0.0466</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.1052 ± 0.0474</t>
+          <t>0.0586 ± 0.0314</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.8953 ± 0.4895</t>
+          <t>0.2676 ± 0.1454</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>44.9282 ± 28.7681</t>
+          <t>14.5499 ± 8.3421</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>month_sin</t>
+          <t>vgo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.0908 ± 0.0607</t>
+          <t>0.0806 ± 0.0545</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.0229 ± 0.0262</t>
+          <t>0.0516 ± 0.0541</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.2619 ± 0.1712</t>
+          <t>0.3448 ± 0.2223</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>15.8797 ± 10.7350</t>
+          <t>14.0690 ± 9.4182</t>
         </is>
       </c>
     </row>
@@ -1248,130 +1248,130 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.0763 ± 0.0587</t>
+          <t>0.0620 ± 0.0247</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.0486 ± 0.0280</t>
+          <t>0.0532 ± 0.0142</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.2820 ± 0.2041</t>
+          <t>0.2474 ± 0.0942</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>13.2842 ± 10.1851</t>
+          <t>10.9005 ± 4.3961</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>mlotst</t>
+          <t>month_sin</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.0458 ± 0.0240</t>
+          <t>0.0540 ± 0.0542</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.0094 ± 0.0303</t>
+          <t>0.0051 ± 0.0187</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.1507 ± 0.0777</t>
+          <t>0.1618 ± 0.1737</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>7.9512 ± 4.1130</t>
+          <t>9.4065 ± 9.4466</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>month_cos</t>
+          <t>to</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0.0239 ± 0.0189</t>
+          <t>0.0183 ± 0.0122</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.0103 ± 0.0133</t>
+          <t>0.0138 ± 0.0212</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.0901 ± 0.0714</t>
+          <t>0.0720 ± 0.0479</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.1795 ± 3.3050</t>
+          <t>3.2008 ± 2.1250</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>to</t>
+          <t>CDM</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.0229 ± 0.0186</t>
+          <t>0.0119 ± 0.0079</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.0103 ± 0.0301</t>
+          <t>0.0079 ± 0.0149</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.0833 ± 0.0725</t>
+          <t>0.0331 ± 0.0262</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4.0193 ± 3.3115</t>
+          <t>2.0812 ± 1.3632</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CDM</t>
+          <t>month_cos</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.0174 ± 0.0145</t>
+          <t>0.0096 ± 0.0102</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-0.0026 ± 0.0119</t>
+          <t>0.0181 ± 0.0161</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.0528 ± 0.0457</t>
+          <t>0.0383 ± 0.0387</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3.0026 ± 2.4805</t>
+          <t>1.6727 ± 1.7650</t>
         </is>
       </c>
     </row>

</xml_diff>